<commit_message>
feat: add character capacity to definition
</commit_message>
<xml_diff>
--- a/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
+++ b/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ThunderbirdsBoardGameEngine\tools\ReferenceData\ThunderbirdsBoardGameEngine.ReferenceData.Compiler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46F7A40A-3752-4C06-83AB-BAFE40D224DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C3D7BBE-A279-4B81-9517-864DB2165C95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Disaster Cards" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="136">
   <si>
     <t>Name</t>
   </si>
@@ -448,6 +448,9 @@
   </si>
   <si>
     <t>Top Speed</t>
+  </si>
+  <si>
+    <t>Character Capacity</t>
   </si>
 </sst>
 </file>
@@ -2234,10 +2237,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0480585C-3CD8-4574-8818-ED7851DE9160}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2247,8 +2250,11 @@
       <c r="C1" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -2258,8 +2264,11 @@
       <c r="C2">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>97</v>
       </c>
@@ -2269,8 +2278,11 @@
       <c r="C3">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>38</v>
       </c>
@@ -2280,8 +2292,11 @@
       <c r="C4">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -2291,8 +2306,11 @@
       <c r="C5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>98</v>
       </c>
@@ -2302,8 +2320,11 @@
       <c r="C6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>33</v>
       </c>
@@ -2312,6 +2333,9 @@
       </c>
       <c r="C7">
         <v>1</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(reference-data): add Thunderbird Machine character capacity (#156)
</commit_message>
<xml_diff>
--- a/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
+++ b/tools/ReferenceData/ThunderbirdsBoardGameEngine.ReferenceData.Compiler/ReferenceData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ThunderbirdsBoardGameEngine\tools\ReferenceData\ThunderbirdsBoardGameEngine.ReferenceData.Compiler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46F7A40A-3752-4C06-83AB-BAFE40D224DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C3D7BBE-A279-4B81-9517-864DB2165C95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{3BAEA212-0460-425E-B252-35BA9C9C29E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Disaster Cards" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="136">
   <si>
     <t>Name</t>
   </si>
@@ -448,6 +448,9 @@
   </si>
   <si>
     <t>Top Speed</t>
+  </si>
+  <si>
+    <t>Character Capacity</t>
   </si>
 </sst>
 </file>
@@ -2234,10 +2237,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0480585C-3CD8-4574-8818-ED7851DE9160}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2247,8 +2250,11 @@
       <c r="C1" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -2258,8 +2264,11 @@
       <c r="C2">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>97</v>
       </c>
@@ -2269,8 +2278,11 @@
       <c r="C3">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>38</v>
       </c>
@@ -2280,8 +2292,11 @@
       <c r="C4">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -2291,8 +2306,11 @@
       <c r="C5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>98</v>
       </c>
@@ -2302,8 +2320,11 @@
       <c r="C6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>33</v>
       </c>
@@ -2312,6 +2333,9 @@
       </c>
       <c r="C7">
         <v>1</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>